<commit_message>
feat(decks): sistema de mazos con validación de cartas y rondas
- agregar tablas tournaments.tournament_registration y
  tournaments.round_deck_selection (faltaban en el modelo original
  para soportar RF-07: inscripción de jugadores a torneos)
- agregar columna quantity a players.deck_card (el catálogo real
  permite copias repetidas de una misma carta, hasta max_quantity)
- modelos SQLAlchemy: TournamentRegistration, RoundDeckSelection
- endpoint players: POST/GET /players/me
- endpoint decks: POST /decks, GET /decks/me,
  POST/GET /decks/{id}/cards (valida max_quantity por carta)
- endpoint tournaments: POST/GET /tournaments/{id}/registrations
- endpoint rounds: POST /rounds/{id}/deck-selection
  (valida mínimo 20 cartas en el mazo antes de permitir selección)
- seed: catálogo real de 18 cartas (cards.card)

fix: eliminar endpoint duplicado en decks.py que causaba que
la cantidad de cartas (quantity) se ignorara siempre
</commit_message>
<xml_diff>
--- a/database/docs/normalizacion.xlsx
+++ b/database/docs/normalizacion.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\santi\Documents\desarrollo_orientado_plataformas\torre-de-cartas\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\santi\Documents\desarrollo_orientado_plataformas\torre-de-cartas\database\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC40E5B4-F1FE-48E6-9088-287E92B33557}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C0567EA-A2A2-491C-9765-93250A492218}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="0FN" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="880" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="885" uniqueCount="198">
   <si>
     <t>FORMA NO NORMALIZADA (0FN)</t>
   </si>
@@ -610,6 +610,18 @@
   </si>
   <si>
     <t>quantity</t>
+  </si>
+  <si>
+    <t>tournament_registration</t>
+  </si>
+  <si>
+    <t>tournament_registration_id</t>
+  </si>
+  <si>
+    <t>tournament_id</t>
+  </si>
+  <si>
+    <t>registered_at</t>
   </si>
 </sst>
 </file>
@@ -847,7 +859,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -987,6 +999,15 @@
     <xf numFmtId="0" fontId="13" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -999,18 +1020,13 @@
     <xf numFmtId="0" fontId="10" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -1857,7 +1873,7 @@
     <mergeCell ref="B2:J2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -5066,9 +5082,10 @@
     <col min="8" max="8" width="24" customWidth="1"/>
     <col min="9" max="9" width="18" customWidth="1"/>
     <col min="10" max="10" width="26.7109375" customWidth="1"/>
-    <col min="11" max="14" width="20" customWidth="1"/>
+    <col min="11" max="13" width="20" customWidth="1"/>
+    <col min="14" max="14" width="25.5703125" customWidth="1"/>
     <col min="15" max="15" width="20.140625" customWidth="1"/>
-    <col min="16" max="16" width="16" customWidth="1"/>
+    <col min="16" max="17" width="16" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:17" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
@@ -5098,7 +5115,7 @@
       <c r="J3" s="43"/>
     </row>
     <row r="5" spans="2:17" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="53" t="s">
+      <c r="B5" s="56" t="s">
         <v>137</v>
       </c>
       <c r="C5" s="42"/>
@@ -5178,24 +5195,24 @@
       </c>
     </row>
     <row r="11" spans="2:17" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="55" t="s">
+      <c r="B11" s="51" t="s">
         <v>145</v>
       </c>
       <c r="C11" s="42"/>
       <c r="D11" s="42"/>
       <c r="E11" s="42"/>
       <c r="F11" s="43"/>
-      <c r="H11" s="56" t="s">
+      <c r="H11" s="52" t="s">
         <v>28</v>
       </c>
       <c r="I11" s="40"/>
       <c r="J11" s="40"/>
       <c r="K11" s="40"/>
-      <c r="M11" s="54" t="s">
+      <c r="M11" s="57" t="s">
         <v>27</v>
       </c>
       <c r="N11" s="43"/>
-      <c r="P11" s="51" t="s">
+      <c r="P11" s="54" t="s">
         <v>146</v>
       </c>
       <c r="Q11" s="43"/>
@@ -5466,7 +5483,7 @@
       <c r="J22" s="2"/>
     </row>
     <row r="23" spans="2:26" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B23" s="55" t="s">
+      <c r="B23" s="51" t="s">
         <v>100</v>
       </c>
       <c r="C23" s="42"/>
@@ -6060,13 +6077,13 @@
       <c r="O38" s="33"/>
     </row>
     <row r="39" spans="2:18" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B39" s="57" t="s">
+      <c r="B39" s="53" t="s">
         <v>2</v>
       </c>
       <c r="C39" s="42"/>
       <c r="D39" s="42"/>
       <c r="E39" s="43"/>
-      <c r="G39" s="52" t="s">
+      <c r="G39" s="55" t="s">
         <v>181</v>
       </c>
       <c r="H39" s="40"/>
@@ -6283,6 +6300,12 @@
       <c r="J47" s="42"/>
       <c r="K47" s="42"/>
       <c r="L47" s="43"/>
+      <c r="N47" s="48" t="s">
+        <v>194</v>
+      </c>
+      <c r="O47" s="48"/>
+      <c r="P47" s="48"/>
+      <c r="Q47" s="48"/>
     </row>
     <row r="48" spans="2:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B48" s="13" t="s">
@@ -6312,8 +6335,20 @@
       <c r="L48" s="15" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="49" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="N48" s="59" t="s">
+        <v>195</v>
+      </c>
+      <c r="O48" s="59" t="s">
+        <v>196</v>
+      </c>
+      <c r="P48" s="59" t="s">
+        <v>96</v>
+      </c>
+      <c r="Q48" s="59" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="49" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B49" s="12">
         <v>1</v>
       </c>
@@ -6337,8 +6372,12 @@
       </c>
       <c r="K49" s="8"/>
       <c r="L49" s="8"/>
-    </row>
-    <row r="50" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="N49" s="60"/>
+      <c r="O49" s="60"/>
+      <c r="P49" s="60"/>
+      <c r="Q49" s="60"/>
+    </row>
+    <row r="50" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B50" s="12">
         <v>2</v>
       </c>
@@ -6362,8 +6401,12 @@
       </c>
       <c r="K50" s="8"/>
       <c r="L50" s="8"/>
-    </row>
-    <row r="51" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="N50" s="60"/>
+      <c r="O50" s="60"/>
+      <c r="P50" s="60"/>
+      <c r="Q50" s="60"/>
+    </row>
+    <row r="51" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B51" s="12">
         <v>3</v>
       </c>
@@ -6387,8 +6430,12 @@
       </c>
       <c r="K51" s="8"/>
       <c r="L51" s="8"/>
-    </row>
-    <row r="52" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="N51" s="60"/>
+      <c r="O51" s="60"/>
+      <c r="P51" s="60"/>
+      <c r="Q51" s="60"/>
+    </row>
+    <row r="52" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B52" s="12">
         <v>4</v>
       </c>
@@ -6412,8 +6459,12 @@
       </c>
       <c r="K52" s="8"/>
       <c r="L52" s="8"/>
-    </row>
-    <row r="53" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="N52" s="60"/>
+      <c r="O52" s="60"/>
+      <c r="P52" s="60"/>
+      <c r="Q52" s="60"/>
+    </row>
+    <row r="53" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B53" s="12">
         <v>5</v>
       </c>
@@ -6437,8 +6488,12 @@
       </c>
       <c r="K53" s="8"/>
       <c r="L53" s="8"/>
-    </row>
-    <row r="54" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="N53" s="60"/>
+      <c r="O53" s="60"/>
+      <c r="P53" s="60"/>
+      <c r="Q53" s="60"/>
+    </row>
+    <row r="54" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B54" s="12">
         <v>6</v>
       </c>
@@ -6462,8 +6517,12 @@
       </c>
       <c r="K54" s="8"/>
       <c r="L54" s="8"/>
-    </row>
-    <row r="55" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="N54" s="60"/>
+      <c r="O54" s="60"/>
+      <c r="P54" s="60"/>
+      <c r="Q54" s="60"/>
+    </row>
+    <row r="55" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B55" s="12">
         <v>7</v>
       </c>
@@ -6487,8 +6546,12 @@
       </c>
       <c r="K55" s="8"/>
       <c r="L55" s="8"/>
-    </row>
-    <row r="56" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="N55" s="60"/>
+      <c r="O55" s="60"/>
+      <c r="P55" s="60"/>
+      <c r="Q55" s="60"/>
+    </row>
+    <row r="56" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B56" s="12">
         <v>8</v>
       </c>
@@ -6512,8 +6575,12 @@
       </c>
       <c r="K56" s="8"/>
       <c r="L56" s="8"/>
-    </row>
-    <row r="57" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="N56" s="60"/>
+      <c r="O56" s="60"/>
+      <c r="P56" s="60"/>
+      <c r="Q56" s="60"/>
+    </row>
+    <row r="57" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B57" s="12">
         <v>9</v>
       </c>
@@ -6530,7 +6597,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="58" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B58" s="12">
         <v>10</v>
       </c>
@@ -6547,7 +6614,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="59" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B59" s="12">
         <v>11</v>
       </c>
@@ -6564,7 +6631,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="60" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B60" s="12">
         <v>12</v>
       </c>
@@ -6582,7 +6649,15 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="15">
+    <mergeCell ref="N47:Q47"/>
+    <mergeCell ref="P11:Q11"/>
+    <mergeCell ref="G39:O39"/>
+    <mergeCell ref="B5:H5"/>
+    <mergeCell ref="B2:J2"/>
+    <mergeCell ref="B3:J3"/>
+    <mergeCell ref="M11:N11"/>
+    <mergeCell ref="P23:R23"/>
     <mergeCell ref="B47:F47"/>
     <mergeCell ref="B23:D23"/>
     <mergeCell ref="B11:F11"/>
@@ -6590,13 +6665,6 @@
     <mergeCell ref="F23:M23"/>
     <mergeCell ref="I47:L47"/>
     <mergeCell ref="B39:E39"/>
-    <mergeCell ref="P11:Q11"/>
-    <mergeCell ref="G39:O39"/>
-    <mergeCell ref="B5:H5"/>
-    <mergeCell ref="B2:J2"/>
-    <mergeCell ref="B3:J3"/>
-    <mergeCell ref="M11:N11"/>
-    <mergeCell ref="P23:R23"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="J13" r:id="rId1" display="mailto:jorge.ortega@gmail.com" xr:uid="{00000000-0004-0000-0300-000000000000}"/>

</xml_diff>